<commit_message>
Täglich: 21.09.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan_daily.xlsx
+++ b/skipperplan_daily.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23500" uniqueCount="2958">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23469" uniqueCount="2957">
   <si>
     <t>Startdatum</t>
   </si>
@@ -8878,9 +8878,6 @@
   </si>
   <si>
     <t>Neue Bewerbungen</t>
-  </si>
-  <si>
-    <t>Neue Bewerbung(en)</t>
   </si>
   <si>
     <t>ID</t>
@@ -10830,7 +10827,7 @@
         <v>9</v>
       </c>
       <c r="J19" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>34</v>
@@ -11536,7 +11533,7 @@
         <v>6</v>
       </c>
       <c r="J28" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>34</v>
@@ -13100,7 +13097,7 @@
         <v>50</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>316</v>
@@ -13180,7 +13177,7 @@
         <v>50</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>323</v>
@@ -13258,7 +13255,7 @@
         <v>50</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>326</v>
@@ -13270,7 +13267,7 @@
         <v>9</v>
       </c>
       <c r="J50" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K50" s="3" t="s">
         <v>34</v>
@@ -13336,7 +13333,7 @@
         <v>50</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>177</v>
@@ -13414,7 +13411,7 @@
         <v>50</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>332</v>
@@ -13492,7 +13489,7 @@
         <v>50</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>336</v>
@@ -15234,7 +15231,7 @@
         <v>9</v>
       </c>
       <c r="J75" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K75" s="5" t="s">
         <v>34</v>
@@ -15938,7 +15935,7 @@
         <v>8</v>
       </c>
       <c r="J84" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K84" s="7" t="s">
         <v>34</v>
@@ -16650,7 +16647,7 @@
         <v>8</v>
       </c>
       <c r="J93" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K93" s="5" t="s">
         <v>34</v>
@@ -18222,7 +18219,7 @@
         <v>8</v>
       </c>
       <c r="J113" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K113" s="6" t="s">
         <v>233</v>
@@ -18770,7 +18767,7 @@
         <v>8</v>
       </c>
       <c r="J120" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K120" s="3" t="s">
         <v>233</v>
@@ -19536,82 +19533,82 @@
       </c>
     </row>
     <row r="130" spans="1:26">
-      <c r="A130" s="6" t="s">
+      <c r="A130" s="7" t="s">
         <v>517</v>
       </c>
-      <c r="B130" s="6" t="s">
+      <c r="B130" s="7" t="s">
         <v>614</v>
       </c>
-      <c r="C130" s="6" t="s">
+      <c r="C130" s="7" t="s">
         <v>531</v>
       </c>
-      <c r="D130" s="6" t="s">
+      <c r="D130" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E130" s="6" t="s">
+      <c r="E130" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F130" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G130" s="6" t="s">
+      <c r="F130" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G130" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="H130" s="6" t="s">
+      <c r="H130" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="I130" s="6">
+      <c r="I130" s="7">
         <v>8</v>
       </c>
-      <c r="J130" s="6">
-        <v>0</v>
-      </c>
-      <c r="K130" s="6" t="s">
+      <c r="J130" s="7">
+        <v>1</v>
+      </c>
+      <c r="K130" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="L130" s="6" t="s">
+      <c r="L130" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="M130" s="6" t="s">
+      <c r="M130" s="7" t="s">
         <v>519</v>
       </c>
-      <c r="N130" s="6" t="s">
+      <c r="N130" s="7" t="s">
         <v>520</v>
       </c>
-      <c r="O130" s="6" t="s">
+      <c r="O130" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="P130" s="6" t="s">
+      <c r="P130" s="7" t="s">
         <v>534</v>
       </c>
-      <c r="Q130" s="6" t="s">
+      <c r="Q130" s="7" t="s">
         <v>627</v>
       </c>
-      <c r="R130" s="6" t="s">
+      <c r="R130" s="7" t="s">
         <v>630</v>
       </c>
-      <c r="S130" s="6" t="s">
+      <c r="S130" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="T130" s="6" t="s">
+      <c r="T130" s="7" t="s">
         <v>537</v>
       </c>
-      <c r="U130" s="6" t="s">
+      <c r="U130" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="V130" s="6">
+      <c r="V130" s="7">
         <v>2016</v>
       </c>
-      <c r="W130" s="6" t="s">
-        <v>473</v>
-      </c>
-      <c r="X130" s="6" t="s">
+      <c r="W130" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="X130" s="7" t="s">
         <v>440</v>
       </c>
-      <c r="Y130" s="6" t="s">
+      <c r="Y130" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="Z130" s="6"/>
+      <c r="Z130" s="7"/>
     </row>
     <row r="131" spans="1:26">
       <c r="A131" s="5" t="s">
@@ -20974,7 +20971,7 @@
         <v>9</v>
       </c>
       <c r="J148" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K148" s="4" t="s">
         <v>233</v>
@@ -21492,7 +21489,7 @@
         <v>45</v>
       </c>
       <c r="X154" s="3" t="s">
-        <v>330</v>
+        <v>290</v>
       </c>
       <c r="Y154" s="3" t="s">
         <v>46</v>
@@ -21604,7 +21601,7 @@
         <v>8</v>
       </c>
       <c r="J156" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K156" s="3" t="s">
         <v>233</v>
@@ -22074,7 +22071,7 @@
         <v>8</v>
       </c>
       <c r="J162" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K162" s="3" t="s">
         <v>233</v>
@@ -29870,7 +29867,7 @@
         <v>12</v>
       </c>
       <c r="J263" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K263" s="7" t="s">
         <v>233</v>
@@ -29946,7 +29943,7 @@
         <v>8</v>
       </c>
       <c r="J264" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K264" s="4" t="s">
         <v>34</v>
@@ -30069,9 +30066,7 @@
       <c r="Y265" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="Z265" s="4" t="s">
-        <v>532</v>
-      </c>
+      <c r="Z265" s="4"/>
     </row>
     <row r="266" spans="1:26">
       <c r="A266" s="4" t="s">
@@ -30332,7 +30327,7 @@
         <v>8</v>
       </c>
       <c r="J269" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K269" s="4" t="s">
         <v>233</v>
@@ -90977,7 +90972,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -91016,121 +91011,6 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>2950</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>552</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>824</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>825</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>561</v>
-      </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>1026</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>1027</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3" t="s">
-        <v>1031</v>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>1037</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>1038</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
-        <v>1041</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>1042</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>1043</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>1043</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>1048</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3" t="s">
-        <v>532</v>
       </c>
     </row>
   </sheetData>
@@ -91156,16 +91036,16 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2951</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2952</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2953</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2954</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2955</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -91182,7 +91062,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -91199,7 +91079,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -91216,7 +91096,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -91233,7 +91113,7 @@
         <v>6</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -91250,7 +91130,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -91267,7 +91147,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -91284,7 +91164,7 @@
         <v>6</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -91301,7 +91181,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -91318,7 +91198,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -91335,7 +91215,7 @@
         <v>8</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -91352,7 +91232,7 @@
         <v>6</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -91369,7 +91249,7 @@
         <v>3</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -91386,7 +91266,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -91403,7 +91283,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -91420,7 +91300,7 @@
         <v>6</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -91437,7 +91317,7 @@
         <v>4</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -91454,7 +91334,7 @@
         <v>4</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -91471,7 +91351,7 @@
         <v>3</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -91488,7 +91368,7 @@
         <v>4</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -91505,7 +91385,7 @@
         <v>3</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -91522,7 +91402,7 @@
         <v>6</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -91539,7 +91419,7 @@
         <v>3</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -91556,7 +91436,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -91573,7 +91453,7 @@
         <v>3</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -91590,7 +91470,7 @@
         <v>2</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -91607,7 +91487,7 @@
         <v>2</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -91624,7 +91504,7 @@
         <v>4</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -91641,7 +91521,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -91658,7 +91538,7 @@
         <v>2</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -91675,7 +91555,7 @@
         <v>3</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -91692,7 +91572,7 @@
         <v>2</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -91709,7 +91589,7 @@
         <v>2</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -91726,7 +91606,7 @@
         <v>2</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -91743,7 +91623,7 @@
         <v>2</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -91760,7 +91640,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -91777,7 +91657,7 @@
         <v>4</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -91794,7 +91674,7 @@
         <v>4</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -91811,7 +91691,7 @@
         <v>1</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -91828,7 +91708,7 @@
         <v>1</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -91845,7 +91725,7 @@
         <v>1</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -91862,7 +91742,7 @@
         <v>1</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -91879,7 +91759,7 @@
         <v>1</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -91896,7 +91776,7 @@
         <v>1</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -91913,7 +91793,7 @@
         <v>1</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -91930,7 +91810,7 @@
         <v>1</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -91947,7 +91827,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -91964,7 +91844,7 @@
         <v>1</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -91981,7 +91861,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -91998,7 +91878,7 @@
         <v>1</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -92015,7 +91895,7 @@
         <v>1</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -92032,7 +91912,7 @@
         <v>1</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -92049,7 +91929,7 @@
         <v>1</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -92066,7 +91946,7 @@
         <v>1</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -92083,7 +91963,7 @@
         <v>1</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -92100,7 +91980,7 @@
         <v>1</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -92117,7 +91997,7 @@
         <v>1</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -92134,7 +92014,7 @@
         <v>1</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -92151,7 +92031,7 @@
         <v>1</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -92168,7 +92048,7 @@
         <v>1</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>2956</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -92185,7 +92065,7 @@
         <v>1</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -92202,7 +92082,7 @@
         <v>1</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -92219,7 +92099,7 @@
         <v>1</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -92236,7 +92116,7 @@
         <v>1</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -92253,7 +92133,7 @@
         <v>1</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -92270,7 +92150,7 @@
         <v>1</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -92287,7 +92167,7 @@
         <v>1</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -92304,7 +92184,7 @@
         <v>1</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -92321,7 +92201,7 @@
         <v>1</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -92338,7 +92218,7 @@
         <v>1</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -92355,7 +92235,7 @@
         <v>2</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -92372,7 +92252,7 @@
         <v>2</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -92389,7 +92269,7 @@
         <v>2</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -92406,7 +92286,7 @@
         <v>2</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -92423,7 +92303,7 @@
         <v>1</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -92440,7 +92320,7 @@
         <v>1</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -92457,7 +92337,7 @@
         <v>2</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -92474,7 +92354,7 @@
         <v>1</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -92491,7 +92371,7 @@
         <v>2</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -92508,7 +92388,7 @@
         <v>2</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -92525,7 +92405,7 @@
         <v>2</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -92542,7 +92422,7 @@
         <v>2</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -92559,7 +92439,7 @@
         <v>2</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -92576,7 +92456,7 @@
         <v>1</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -92593,7 +92473,7 @@
         <v>2</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -92610,7 +92490,7 @@
         <v>2</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -92627,7 +92507,7 @@
         <v>2</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -92644,7 +92524,7 @@
         <v>2</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -92661,7 +92541,7 @@
         <v>2</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -92678,7 +92558,7 @@
         <v>2</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>2957</v>
+        <v>2956</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Täglich: 25.09.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan_daily.xlsx
+++ b/skipperplan_daily.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23531" uniqueCount="2959">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23511" uniqueCount="2958">
   <si>
     <t>Startdatum</t>
   </si>
@@ -2091,7 +2091,7 @@
     <t>16719</t>
   </si>
   <si>
-    <t>Ralf B, Hendrik B</t>
+    <t>Ralf B, Hendrik B, Julia H</t>
   </si>
   <si>
     <t>09.01.2027</t>
@@ -2589,7 +2589,7 @@
     <t>JEREZ</t>
   </si>
   <si>
-    <t>Andreas N, Michele A, Viktoria B, Aaron B</t>
+    <t>Andreas N, Michele A, Viktoria B, Aaron B, Julia H</t>
   </si>
   <si>
     <t>16734</t>
@@ -2682,7 +2682,7 @@
     <t>16735</t>
   </si>
   <si>
-    <t>Sebastian S, Viktoria B, Florian B, Jan J, Sarin G</t>
+    <t>Sebastian S, Viktoria B, Florian B, Jan J, Sarin G, Julia H</t>
   </si>
   <si>
     <t>16736</t>
@@ -8881,9 +8881,6 @@
   </si>
   <si>
     <t>Neue Bewerbung(en)</t>
-  </si>
-  <si>
-    <t>Neues Boot</t>
   </si>
   <si>
     <t>ID</t>
@@ -8937,7 +8934,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8982,12 +8979,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -9020,7 +9011,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -9043,13 +9034,10 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10592,7 +10580,7 @@
         <v>30</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>144</v>
@@ -10672,7 +10660,7 @@
         <v>30</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>150</v>
@@ -10750,7 +10738,7 @@
         <v>30</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>155</v>
@@ -10828,7 +10816,7 @@
         <v>30</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>160</v>
@@ -12176,7 +12164,7 @@
         <v>8</v>
       </c>
       <c r="J36" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K36" s="3" t="s">
         <v>34</v>
@@ -13030,7 +13018,7 @@
         <v>30</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>307</v>
@@ -13110,7 +13098,7 @@
         <v>30</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>314</v>
@@ -13188,7 +13176,7 @@
         <v>30</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>317</v>
@@ -13266,7 +13254,7 @@
         <v>30</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>167</v>
@@ -13344,7 +13332,7 @@
         <v>30</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>323</v>
@@ -13422,7 +13410,7 @@
         <v>30</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>327</v>
@@ -14027,7 +14015,7 @@
         <v>45</v>
       </c>
       <c r="Y59" s="5" t="s">
-        <v>46</v>
+        <v>200</v>
       </c>
       <c r="Z59" s="5"/>
     </row>
@@ -15072,7 +15060,7 @@
         <v>30</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G73" s="5" t="s">
         <v>124</v>
@@ -15152,7 +15140,7 @@
         <v>30</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G74" s="3" t="s">
         <v>404</v>
@@ -15230,7 +15218,7 @@
         <v>30</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G75" s="5" t="s">
         <v>195</v>
@@ -15242,7 +15230,7 @@
         <v>8</v>
       </c>
       <c r="J75" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K75" s="5" t="s">
         <v>34</v>
@@ -16568,7 +16556,7 @@
         <v>30</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>459</v>
@@ -16648,7 +16636,7 @@
         <v>30</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G93" s="6" t="s">
         <v>464</v>
@@ -16726,7 +16714,7 @@
         <v>30</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>124</v>
@@ -16974,7 +16962,7 @@
         <v>8</v>
       </c>
       <c r="J97" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K97" s="5" t="s">
         <v>34</v>
@@ -18072,7 +18060,7 @@
         <v>8</v>
       </c>
       <c r="J111" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K111" s="6" t="s">
         <v>223</v>
@@ -19004,7 +18992,7 @@
         <v>544</v>
       </c>
       <c r="F123" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G123" s="5" t="s">
         <v>545</v>
@@ -19096,7 +19084,7 @@
         <v>12</v>
       </c>
       <c r="J124" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K124" s="3" t="s">
         <v>223</v>
@@ -19414,7 +19402,7 @@
         <v>8</v>
       </c>
       <c r="J128" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K128" s="7" t="s">
         <v>223</v>
@@ -21690,7 +21678,7 @@
         <v>8</v>
       </c>
       <c r="J157" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K157" s="5" t="s">
         <v>223</v>
@@ -22458,7 +22446,7 @@
         <v>544</v>
       </c>
       <c r="F167" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G167" s="5" t="s">
         <v>359</v>
@@ -22538,7 +22526,7 @@
         <v>544</v>
       </c>
       <c r="F168" s="3" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G168" s="3" t="s">
         <v>766</v>
@@ -22616,7 +22604,7 @@
         <v>544</v>
       </c>
       <c r="F169" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G169" s="5" t="s">
         <v>201</v>
@@ -23170,7 +23158,7 @@
         <v>8</v>
       </c>
       <c r="J176" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K176" s="3" t="s">
         <v>223</v>
@@ -24162,7 +24150,7 @@
         <v>220</v>
       </c>
       <c r="F189" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G189" s="4" t="s">
         <v>502</v>
@@ -24240,7 +24228,7 @@
         <v>220</v>
       </c>
       <c r="F190" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G190" s="4" t="s">
         <v>502</v>
@@ -24316,7 +24304,7 @@
         <v>220</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G191" s="4" t="s">
         <v>502</v>
@@ -24470,7 +24458,7 @@
         <v>220</v>
       </c>
       <c r="F193" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G193" s="5" t="s">
         <v>359</v>
@@ -24550,7 +24538,7 @@
         <v>220</v>
       </c>
       <c r="F194" s="6" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G194" s="6" t="s">
         <v>502</v>
@@ -24626,7 +24614,7 @@
         <v>220</v>
       </c>
       <c r="F195" s="5" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G195" s="5" t="s">
         <v>842</v>
@@ -24704,7 +24692,7 @@
         <v>220</v>
       </c>
       <c r="F196" s="7" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G196" s="7" t="s">
         <v>846</v>
@@ -24782,7 +24770,7 @@
         <v>220</v>
       </c>
       <c r="F197" s="6" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G197" s="6" t="s">
         <v>502</v>
@@ -26168,7 +26156,7 @@
         <v>544</v>
       </c>
       <c r="F215" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G215" s="4" t="s">
         <v>502</v>
@@ -26246,7 +26234,7 @@
         <v>544</v>
       </c>
       <c r="F216" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G216" s="4" t="s">
         <v>502</v>
@@ -26322,7 +26310,7 @@
         <v>544</v>
       </c>
       <c r="F217" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G217" s="4" t="s">
         <v>502</v>
@@ -28550,7 +28538,7 @@
         <v>30</v>
       </c>
       <c r="F246" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G246" s="4" t="s">
         <v>502</v>
@@ -28628,7 +28616,7 @@
         <v>30</v>
       </c>
       <c r="F247" s="4" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G247" s="4" t="s">
         <v>502</v>
@@ -91061,7 +91049,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -91107,22 +91095,22 @@
         <v>2951</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>574</v>
+        <v>612</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>556</v>
+        <v>674</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>557</v>
+        <v>685</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
-        <v>578</v>
+        <v>616</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3" t="s">
-        <v>1686</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -91133,115 +91121,42 @@
         <v>634</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>557</v>
+        <v>827</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>605</v>
+        <v>801</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
-        <v>640</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>662</v>
-      </c>
+        <v>853</v>
+      </c>
+      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
-        <v>1210</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="8" t="s">
-        <v>2952</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>522</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>674</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>689</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>538</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>696</v>
-      </c>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="3" t="s">
+      <c r="A4" s="3" t="s">
         <v>2951</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>757</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>758</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>600</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>777</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
-        <v>552</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3" t="s">
-        <v>1210</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="3" t="s">
-        <v>2951</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>858</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>859</v>
-      </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3" t="s">
-        <v>430</v>
+      <c r="B4" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -91267,1563 +91182,1563 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2952</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2953</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2954</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2955</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2956</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>951</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>6</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>8</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>2957</v>
+      <c r="E2" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="10">
         <v>26133</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="10">
         <v>6</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="10">
         <v>8</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>13707</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>5</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>5</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>2957</v>
+      <c r="E4" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <v>14111</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="10">
         <v>5</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="10">
         <v>6</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>2957</v>
+      <c r="E5" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>13045</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>4</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>6</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <v>13035</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <v>4</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="10">
         <v>5</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>2957</v>
+      <c r="E7" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>15339</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="8">
         <v>4</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="8">
         <v>6</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <v>6429</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="10">
         <v>4</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="10">
         <v>6</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>2957</v>
+      <c r="E9" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
         <v>545</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>26767</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>4</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>8</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <v>27366</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="10">
         <v>3</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="10">
         <v>6</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>22825</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>3</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>3</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <v>9630</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="10">
         <v>3</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="10">
         <v>3</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>17277</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>3</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>6</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>2957</v>
+      <c r="E14" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <v>38249</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="10">
         <v>3</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="10">
         <v>4</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>25998</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>3</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="8">
         <v>4</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <v>27191</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="10">
         <v>3</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="10">
         <v>3</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>28325</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>3</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>4</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>2957</v>
+      <c r="E18" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <v>27428</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="10">
         <v>3</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="10">
         <v>3</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="3" t="s">
         <v>567</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>38409</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>3</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>6</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <v>36958</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="10">
         <v>2</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <v>2</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="8">
         <v>18683</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="8">
         <v>2</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="8">
         <v>3</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <v>2430</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="10">
         <v>2</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <v>2</v>
       </c>
-      <c r="E23" s="10" t="s">
-        <v>2957</v>
+      <c r="E23" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="8">
         <v>44643</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="8">
         <v>2</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="8">
         <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="10">
         <v>14767</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="10">
         <v>2</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <v>3</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="8">
         <v>31914</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="8">
         <v>2</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="10">
         <v>20147</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="10">
         <v>2</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="10">
         <v>4</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>2957</v>
+      <c r="E27" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>6758</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="8">
         <v>2</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="8">
         <v>4</v>
       </c>
-      <c r="E28" s="10" t="s">
-        <v>2957</v>
+      <c r="E28" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="10">
         <v>21701</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="10">
         <v>2</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="10">
         <v>2</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="8">
         <v>17056</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="8">
         <v>2</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="8">
         <v>3</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="10">
         <v>3641</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="10">
         <v>2</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="10">
         <v>2</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="8">
         <v>3223</v>
       </c>
-      <c r="C32" s="9">
+      <c r="C32" s="8">
         <v>2</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="8">
         <v>2</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="10">
         <v>7022</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="10">
         <v>2</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="10">
         <v>2</v>
       </c>
-      <c r="E33" s="10" t="s">
-        <v>2957</v>
+      <c r="E33" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="8">
         <v>27634</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="8">
         <v>2</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="8">
         <v>2</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="10">
         <v>27871</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="10">
         <v>2</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D35" s="10">
         <v>2</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <v>2257</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="8">
         <v>2</v>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="8">
         <v>4</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="10">
         <v>25583</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="10">
         <v>2</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D37" s="10">
         <v>4</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="3" t="s">
         <v>624</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="8">
         <v>27408</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="8">
         <v>2</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="8">
         <v>2</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="5" t="s">
         <v>783</v>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="10">
         <v>27030</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="10">
         <v>2</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D39" s="10">
         <v>4</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="8">
         <v>20508</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="8">
         <v>1</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="8">
         <v>1</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="10">
         <v>17023</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="10">
         <v>1</v>
       </c>
-      <c r="D41" s="11">
+      <c r="D41" s="10">
         <v>1</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="8">
         <v>19061</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="8">
         <v>1</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="8">
         <v>1</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="10">
         <v>28683</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="10">
         <v>1</v>
       </c>
-      <c r="D43" s="11">
+      <c r="D43" s="10">
         <v>1</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="8">
         <v>26955</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="8">
         <v>1</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="8">
         <v>1</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="10">
         <v>23794</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="10">
         <v>1</v>
       </c>
-      <c r="D45" s="11">
+      <c r="D45" s="10">
         <v>1</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="8">
         <v>5432</v>
       </c>
-      <c r="C46" s="9">
+      <c r="C46" s="8">
         <v>1</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="8">
         <v>1</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="10">
         <v>16471</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="10">
         <v>1</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D47" s="10">
         <v>1</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="8">
         <v>10551</v>
       </c>
-      <c r="C48" s="9">
+      <c r="C48" s="8">
         <v>1</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="8">
         <v>1</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="10">
         <v>13592</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="10">
         <v>1</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="10">
         <v>1</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="8">
         <v>39495</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C50" s="8">
         <v>1</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50" s="8">
         <v>1</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="10">
         <v>6756</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="10">
         <v>1</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D51" s="10">
         <v>1</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="8">
         <v>23628</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52" s="8">
         <v>1</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="8">
         <v>1</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="10">
         <v>37876</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="10">
         <v>1</v>
       </c>
-      <c r="D53" s="11">
+      <c r="D53" s="10">
         <v>1</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="8">
         <v>30709</v>
       </c>
-      <c r="C54" s="9">
+      <c r="C54" s="8">
         <v>1</v>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="8">
         <v>1</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="10">
         <v>22942</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="10">
         <v>1</v>
       </c>
-      <c r="D55" s="11">
+      <c r="D55" s="10">
         <v>1</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="8">
         <v>16666</v>
       </c>
-      <c r="C56" s="9">
+      <c r="C56" s="8">
         <v>1</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="8">
         <v>1</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="10">
         <v>12024</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="10">
         <v>1</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="10">
         <v>1</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="8">
         <v>51089</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="8">
         <v>1</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="8">
         <v>1</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="B59" s="11">
+      <c r="B59" s="10">
         <v>27342</v>
       </c>
-      <c r="C59" s="11">
+      <c r="C59" s="10">
         <v>1</v>
       </c>
-      <c r="D59" s="11">
+      <c r="D59" s="10">
         <v>1</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="8">
         <v>2866</v>
       </c>
-      <c r="C60" s="9">
+      <c r="C60" s="8">
         <v>1</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="8">
         <v>1</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="B61" s="11">
+      <c r="B61" s="10">
         <v>17561</v>
       </c>
-      <c r="C61" s="11">
+      <c r="C61" s="10">
         <v>1</v>
       </c>
-      <c r="D61" s="11">
+      <c r="D61" s="10">
         <v>1</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="8">
         <v>347</v>
       </c>
-      <c r="C62" s="9">
+      <c r="C62" s="8">
         <v>1</v>
       </c>
-      <c r="D62" s="9">
+      <c r="D62" s="8">
         <v>1</v>
       </c>
-      <c r="E62" s="10" t="s">
-        <v>2957</v>
+      <c r="E62" s="9" t="s">
+        <v>2956</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="B63" s="11">
+      <c r="B63" s="10">
         <v>22102</v>
       </c>
-      <c r="C63" s="11">
+      <c r="C63" s="10">
         <v>1</v>
       </c>
-      <c r="D63" s="11">
+      <c r="D63" s="10">
         <v>1</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="8">
         <v>25322</v>
       </c>
-      <c r="C64" s="9">
+      <c r="C64" s="8">
         <v>1</v>
       </c>
-      <c r="D64" s="9">
+      <c r="D64" s="8">
         <v>1</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="B65" s="11">
+      <c r="B65" s="10">
         <v>24701</v>
       </c>
-      <c r="C65" s="11">
+      <c r="C65" s="10">
         <v>1</v>
       </c>
-      <c r="D65" s="11">
+      <c r="D65" s="10">
         <v>1</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="8">
         <v>11122</v>
       </c>
-      <c r="C66" s="9">
+      <c r="C66" s="8">
         <v>1</v>
       </c>
-      <c r="D66" s="9">
+      <c r="D66" s="8">
         <v>1</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="B67" s="11">
+      <c r="B67" s="10">
         <v>4911</v>
       </c>
-      <c r="C67" s="11">
+      <c r="C67" s="10">
         <v>1</v>
       </c>
-      <c r="D67" s="11">
+      <c r="D67" s="10">
         <v>1</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="B68" s="9">
+      <c r="B68" s="8">
         <v>25299</v>
       </c>
-      <c r="C68" s="9">
+      <c r="C68" s="8">
         <v>1</v>
       </c>
-      <c r="D68" s="9">
+      <c r="D68" s="8">
         <v>1</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="5" t="s">
         <v>443</v>
       </c>
-      <c r="B69" s="11">
+      <c r="B69" s="10">
         <v>12209</v>
       </c>
-      <c r="C69" s="11">
+      <c r="C69" s="10">
         <v>1</v>
       </c>
-      <c r="D69" s="11">
+      <c r="D69" s="10">
         <v>1</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="B70" s="9">
+      <c r="B70" s="8">
         <v>14124</v>
       </c>
-      <c r="C70" s="9">
+      <c r="C70" s="8">
         <v>1</v>
       </c>
-      <c r="D70" s="9">
+      <c r="D70" s="8">
         <v>1</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="5" t="s">
         <v>459</v>
       </c>
-      <c r="B71" s="11">
+      <c r="B71" s="10">
         <v>13834</v>
       </c>
-      <c r="C71" s="11">
+      <c r="C71" s="10">
         <v>1</v>
       </c>
-      <c r="D71" s="11">
+      <c r="D71" s="10">
         <v>1</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="B72" s="9">
+      <c r="B72" s="8">
         <v>763</v>
       </c>
-      <c r="C72" s="9">
+      <c r="C72" s="8">
         <v>1</v>
       </c>
-      <c r="D72" s="9">
+      <c r="D72" s="8">
         <v>1</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="5" t="s">
         <v>523</v>
       </c>
-      <c r="B73" s="11">
+      <c r="B73" s="10">
         <v>23061</v>
       </c>
-      <c r="C73" s="11">
+      <c r="C73" s="10">
         <v>1</v>
       </c>
-      <c r="D73" s="11">
+      <c r="D73" s="10">
         <v>2</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" s="3" t="s">
         <v>532</v>
       </c>
-      <c r="B74" s="9">
+      <c r="B74" s="8">
         <v>19891</v>
       </c>
-      <c r="C74" s="9">
+      <c r="C74" s="8">
         <v>1</v>
       </c>
-      <c r="D74" s="9">
+      <c r="D74" s="8">
         <v>2</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="5" t="s">
         <v>559</v>
       </c>
-      <c r="B75" s="11">
+      <c r="B75" s="10">
         <v>5443</v>
       </c>
-      <c r="C75" s="11">
+      <c r="C75" s="10">
         <v>1</v>
       </c>
-      <c r="D75" s="11">
+      <c r="D75" s="10">
         <v>2</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" s="3" t="s">
         <v>595</v>
       </c>
-      <c r="B76" s="9">
+      <c r="B76" s="8">
         <v>9849</v>
       </c>
-      <c r="C76" s="9">
+      <c r="C76" s="8">
         <v>1</v>
       </c>
-      <c r="D76" s="9">
+      <c r="D76" s="8">
         <v>2</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" s="5" t="s">
         <v>635</v>
       </c>
-      <c r="B77" s="11">
+      <c r="B77" s="10">
         <v>5205</v>
       </c>
-      <c r="C77" s="11">
+      <c r="C77" s="10">
         <v>1</v>
       </c>
-      <c r="D77" s="11">
+      <c r="D77" s="10">
         <v>1</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" s="3" t="s">
         <v>642</v>
       </c>
-      <c r="B78" s="9">
+      <c r="B78" s="8">
         <v>14023</v>
       </c>
-      <c r="C78" s="9">
+      <c r="C78" s="8">
         <v>1</v>
       </c>
-      <c r="D78" s="9">
+      <c r="D78" s="8">
         <v>1</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="5" t="s">
         <v>649</v>
       </c>
-      <c r="B79" s="11">
+      <c r="B79" s="10">
         <v>6935</v>
       </c>
-      <c r="C79" s="11">
+      <c r="C79" s="10">
         <v>1</v>
       </c>
-      <c r="D79" s="11">
+      <c r="D79" s="10">
         <v>2</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" s="3" t="s">
         <v>662</v>
       </c>
-      <c r="B80" s="9">
+      <c r="B80" s="8">
         <v>27276</v>
       </c>
-      <c r="C80" s="9">
+      <c r="C80" s="8">
         <v>1</v>
       </c>
-      <c r="D80" s="9">
+      <c r="D80" s="8">
         <v>1</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" s="5" t="s">
         <v>690</v>
       </c>
-      <c r="B81" s="11">
+      <c r="B81" s="10">
         <v>12507</v>
       </c>
-      <c r="C81" s="11">
+      <c r="C81" s="10">
         <v>1</v>
       </c>
-      <c r="D81" s="11">
+      <c r="D81" s="10">
         <v>2</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="3" t="s">
         <v>701</v>
       </c>
-      <c r="B82" s="9">
+      <c r="B82" s="8">
         <v>27838</v>
       </c>
-      <c r="C82" s="9">
+      <c r="C82" s="8">
         <v>1</v>
       </c>
-      <c r="D82" s="9">
+      <c r="D82" s="8">
         <v>2</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="5" t="s">
         <v>722</v>
       </c>
-      <c r="B83" s="11">
+      <c r="B83" s="10">
         <v>38991</v>
       </c>
-      <c r="C83" s="11">
+      <c r="C83" s="10">
         <v>1</v>
       </c>
-      <c r="D83" s="11">
+      <c r="D83" s="10">
         <v>2</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" s="3" t="s">
         <v>726</v>
       </c>
-      <c r="B84" s="9">
+      <c r="B84" s="8">
         <v>23196</v>
       </c>
-      <c r="C84" s="9">
+      <c r="C84" s="8">
         <v>1</v>
       </c>
-      <c r="D84" s="9">
+      <c r="D84" s="8">
         <v>2</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" s="5" t="s">
         <v>737</v>
       </c>
-      <c r="B85" s="11">
+      <c r="B85" s="10">
         <v>18695</v>
       </c>
-      <c r="C85" s="11">
+      <c r="C85" s="10">
         <v>1</v>
       </c>
-      <c r="D85" s="11">
+      <c r="D85" s="10">
         <v>2</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" s="3" t="s">
         <v>748</v>
       </c>
-      <c r="B86" s="9">
+      <c r="B86" s="8">
         <v>11162</v>
       </c>
-      <c r="C86" s="9">
+      <c r="C86" s="8">
         <v>1</v>
       </c>
-      <c r="D86" s="9">
+      <c r="D86" s="8">
         <v>1</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="87" spans="1:5">
       <c r="A87" s="5" t="s">
         <v>766</v>
       </c>
-      <c r="B87" s="11">
+      <c r="B87" s="10">
         <v>14252</v>
       </c>
-      <c r="C87" s="11">
+      <c r="C87" s="10">
         <v>1</v>
       </c>
-      <c r="D87" s="11">
+      <c r="D87" s="10">
         <v>2</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" s="3" t="s">
         <v>796</v>
       </c>
-      <c r="B88" s="9">
+      <c r="B88" s="8">
         <v>26388</v>
       </c>
-      <c r="C88" s="9">
+      <c r="C88" s="8">
         <v>1</v>
       </c>
-      <c r="D88" s="9">
+      <c r="D88" s="8">
         <v>2</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" s="5" t="s">
         <v>842</v>
       </c>
-      <c r="B89" s="11">
+      <c r="B89" s="10">
         <v>26443</v>
       </c>
-      <c r="C89" s="11">
+      <c r="C89" s="10">
         <v>1</v>
       </c>
-      <c r="D89" s="11">
+      <c r="D89" s="10">
         <v>2</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="90" spans="1:5">
       <c r="A90" s="3" t="s">
         <v>846</v>
       </c>
-      <c r="B90" s="9">
+      <c r="B90" s="8">
         <v>7195</v>
       </c>
-      <c r="C90" s="9">
+      <c r="C90" s="8">
         <v>1</v>
       </c>
-      <c r="D90" s="9">
+      <c r="D90" s="8">
         <v>2</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="91" spans="1:5">
       <c r="A91" s="5" t="s">
         <v>985</v>
       </c>
-      <c r="B91" s="11">
+      <c r="B91" s="10">
         <v>5335</v>
       </c>
-      <c r="C91" s="11">
+      <c r="C91" s="10">
         <v>1</v>
       </c>
-      <c r="D91" s="11">
+      <c r="D91" s="10">
         <v>2</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="92" spans="1:5">
       <c r="A92" s="3" t="s">
         <v>991</v>
       </c>
-      <c r="B92" s="9">
+      <c r="B92" s="8">
         <v>19273</v>
       </c>
-      <c r="C92" s="9">
+      <c r="C92" s="8">
         <v>1</v>
       </c>
-      <c r="D92" s="9">
+      <c r="D92" s="8">
         <v>2</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>2958</v>
+        <v>2957</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Täglich: 28.09.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan_daily.xlsx
+++ b/skipperplan_daily.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23506" uniqueCount="2963">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23499" uniqueCount="2962">
   <si>
     <t>Startdatum</t>
   </si>
@@ -8893,9 +8893,6 @@
   </si>
   <si>
     <t>Neue Bewerbungen</t>
-  </si>
-  <si>
-    <t>Neue Bewerbung(en)</t>
   </si>
   <si>
     <t>ID</t>
@@ -16741,7 +16738,7 @@
         <v>7</v>
       </c>
       <c r="J94" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K94" s="3" t="s">
         <v>263</v>
@@ -18151,7 +18148,7 @@
         <v>8</v>
       </c>
       <c r="J112" s="6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K112" s="6" t="s">
         <v>263</v>
@@ -18859,7 +18856,7 @@
         <v>8</v>
       </c>
       <c r="J121" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K121" s="5" t="s">
         <v>263</v>
@@ -19405,7 +19402,7 @@
         <v>9</v>
       </c>
       <c r="J128" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K128" s="3" t="s">
         <v>263</v>
@@ -20339,7 +20336,7 @@
         <v>8</v>
       </c>
       <c r="J140" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K140" s="3" t="s">
         <v>263</v>
@@ -27273,7 +27270,7 @@
         <v>10</v>
       </c>
       <c r="J230" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K230" s="4" t="s">
         <v>34</v>
@@ -91178,7 +91175,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -91217,31 +91214,6 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>2955</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="3" t="s">
-        <v>2956</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>501</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>472</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>529</v>
-      </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
-        <v>1304</v>
       </c>
     </row>
   </sheetData>
@@ -91267,16 +91239,16 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2956</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2957</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2958</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2959</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2960</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -91293,7 +91265,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -91310,7 +91282,7 @@
         <v>7</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -91327,7 +91299,7 @@
         <v>6</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -91344,7 +91316,7 @@
         <v>4</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -91361,7 +91333,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -91378,7 +91350,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -91395,7 +91367,7 @@
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -91412,7 +91384,7 @@
         <v>3</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -91429,7 +91401,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -91446,7 +91418,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -91463,7 +91435,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -91480,7 +91452,7 @@
         <v>4</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -91497,7 +91469,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -91514,7 +91486,7 @@
         <v>6</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -91531,7 +91503,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -91548,7 +91520,7 @@
         <v>2</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -91565,7 +91537,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -91582,7 +91554,7 @@
         <v>2</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -91599,7 +91571,7 @@
         <v>3</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -91616,7 +91588,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -91633,7 +91605,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -91650,7 +91622,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -91667,7 +91639,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -91684,7 +91656,7 @@
         <v>4</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -91701,7 +91673,7 @@
         <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -91718,7 +91690,7 @@
         <v>4</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -91735,7 +91707,7 @@
         <v>4</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -91752,7 +91724,7 @@
         <v>2</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -91769,7 +91741,7 @@
         <v>4</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -91786,7 +91758,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -91803,7 +91775,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -91820,7 +91792,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -91837,7 +91809,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -91854,7 +91826,7 @@
         <v>1</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -91871,7 +91843,7 @@
         <v>1</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -91888,7 +91860,7 @@
         <v>1</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -91905,7 +91877,7 @@
         <v>1</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -91922,7 +91894,7 @@
         <v>1</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -91939,7 +91911,7 @@
         <v>1</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -91956,7 +91928,7 @@
         <v>1</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -91973,7 +91945,7 @@
         <v>1</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -91990,7 +91962,7 @@
         <v>1</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -92007,7 +91979,7 @@
         <v>1</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -92024,7 +91996,7 @@
         <v>2</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -92041,7 +92013,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -92058,7 +92030,7 @@
         <v>2</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>2962</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -92075,7 +92047,7 @@
         <v>1</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -92092,7 +92064,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -92109,7 +92081,7 @@
         <v>1</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -92126,7 +92098,7 @@
         <v>1</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -92143,7 +92115,7 @@
         <v>1</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -92160,7 +92132,7 @@
         <v>1</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -92177,7 +92149,7 @@
         <v>2</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -92194,7 +92166,7 @@
         <v>2</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -92211,7 +92183,7 @@
         <v>2</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -92228,7 +92200,7 @@
         <v>2</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -92245,7 +92217,7 @@
         <v>2</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -92262,7 +92234,7 @@
         <v>1</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -92279,7 +92251,7 @@
         <v>1</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -92296,7 +92268,7 @@
         <v>2</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -92313,7 +92285,7 @@
         <v>1</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -92330,7 +92302,7 @@
         <v>2</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -92347,7 +92319,7 @@
         <v>2</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -92364,7 +92336,7 @@
         <v>2</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -92381,7 +92353,7 @@
         <v>2</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -92398,7 +92370,7 @@
         <v>2</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -92415,7 +92387,7 @@
         <v>1</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -92432,7 +92404,7 @@
         <v>2</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -92449,7 +92421,7 @@
         <v>2</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -92466,7 +92438,7 @@
         <v>2</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -92483,7 +92455,7 @@
         <v>2</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -92500,7 +92472,7 @@
         <v>2</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -92517,7 +92489,7 @@
         <v>2</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -92534,7 +92506,7 @@
         <v>2</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>2961</v>
+        <v>2960</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Täglich: 30.09.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan_daily.xlsx
+++ b/skipperplan_daily.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23551" uniqueCount="2967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23499" uniqueCount="2963">
   <si>
     <t>Startdatum</t>
   </si>
@@ -8896,18 +8896,6 @@
   </si>
   <si>
     <t>Neue Bewerbungen</t>
-  </si>
-  <si>
-    <t>Skipper geändert</t>
-  </si>
-  <si>
-    <t>Neues Boot</t>
-  </si>
-  <si>
-    <t>Storniert</t>
-  </si>
-  <si>
-    <t>Angelo</t>
   </si>
   <si>
     <t>ID</t>
@@ -8961,7 +8949,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9006,18 +8994,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -9050,7 +9026,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -9073,19 +9049,13 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -15271,7 +15241,7 @@
         <v>8</v>
       </c>
       <c r="J75" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K75" s="6" t="s">
         <v>265</v>
@@ -16613,7 +16583,7 @@
         <v>8</v>
       </c>
       <c r="J92" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K92" s="7" t="s">
         <v>265</v>
@@ -18181,7 +18151,7 @@
         <v>8</v>
       </c>
       <c r="J112" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>265</v>
@@ -18651,7 +18621,7 @@
         <v>8</v>
       </c>
       <c r="J118" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K118" s="6" t="s">
         <v>265</v>
@@ -18889,7 +18859,7 @@
         <v>8</v>
       </c>
       <c r="J121" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K121" s="5" t="s">
         <v>265</v>
@@ -19201,7 +19171,7 @@
         <v>8</v>
       </c>
       <c r="J125" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K125" s="4" t="s">
         <v>265</v>
@@ -27611,7 +27581,7 @@
         <v>8</v>
       </c>
       <c r="J234" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K234" s="4" t="s">
         <v>265</v>
@@ -91208,7 +91178,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -91248,187 +91218,6 @@
       <c r="I1" s="1" t="s">
         <v>2956</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="8" t="s">
-        <v>2957</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="I2" s="8"/>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="8" t="s">
-        <v>2957</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="I3" s="8"/>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="8" t="s">
-        <v>2957</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="8" t="s">
-        <v>2957</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>337</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="I5" s="8"/>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="8" t="s">
-        <v>2957</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>337</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="I6" s="8"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="9" t="s">
-        <v>2958</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>386</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>543</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>558</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>583</v>
-      </c>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="7" t="s">
-        <v>2959</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>386</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>543</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>558</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>2960</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -91453,1274 +91242,1274 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2961</v>
+        <v>2957</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2962</v>
+        <v>2958</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2963</v>
+        <v>2959</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2964</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="8">
         <v>26133</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="8">
         <v>6</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="8">
         <v>8</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="9">
         <v>951</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="9">
         <v>5</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="9">
         <v>7</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>2966</v>
+      <c r="E3" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>14111</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>5</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>6</v>
       </c>
-      <c r="E4" s="12" t="s">
-        <v>2966</v>
+      <c r="E4" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="9">
         <v>13707</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="9">
         <v>4</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="9">
         <v>4</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>2966</v>
+      <c r="E5" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>6429</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>4</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>6</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>2966</v>
+      <c r="E6" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="9">
         <v>26767</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="9">
         <v>4</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="9">
         <v>8</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="8">
         <v>25998</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="8">
         <v>3</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="8">
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="9">
         <v>27191</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="9">
         <v>3</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="9">
         <v>3</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="8">
         <v>15339</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <v>3</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="8">
         <v>5</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="9">
         <v>13035</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="9">
         <v>3</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="9">
         <v>4</v>
       </c>
-      <c r="E11" s="12" t="s">
-        <v>2966</v>
+      <c r="E11" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="8">
         <v>13045</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <v>3</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="8">
         <v>5</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="9">
         <v>28325</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="9">
         <v>3</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="9">
         <v>4</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>2966</v>
+      <c r="E13" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="8">
         <v>27428</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <v>3</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="9">
         <v>38409</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="9">
         <v>3</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="9">
         <v>6</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="8">
         <v>17056</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <v>2</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="8">
         <v>3</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="9">
         <v>22825</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="9">
         <v>2</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="9">
         <v>2</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>3641</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>2</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>2</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="9">
         <v>3223</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="9">
         <v>2</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="9">
         <v>2</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>38249</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>2</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>3</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="9">
         <v>7022</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="9">
         <v>2</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="9">
         <v>2</v>
       </c>
-      <c r="E21" s="12" t="s">
-        <v>2966</v>
+      <c r="E21" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="8">
         <v>27634</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C22" s="8">
         <v>2</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="8">
         <v>2</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="9">
         <v>9630</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="9">
         <v>2</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="9">
         <v>2</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="8">
         <v>27871</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <v>2</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="8">
         <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="9">
         <v>17277</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="9">
         <v>2</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="9">
         <v>4</v>
       </c>
-      <c r="E25" s="12" t="s">
-        <v>2966</v>
+      <c r="E25" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>2257</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>2</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="9">
         <v>27366</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="9">
         <v>2</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="9">
         <v>4</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="8">
         <v>25583</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="8">
         <v>2</v>
       </c>
-      <c r="D28" s="10">
+      <c r="D28" s="8">
         <v>4</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="5" t="s">
         <v>493</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="9">
         <v>27408</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="9">
         <v>2</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="9">
         <v>2</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="3" t="s">
         <v>655</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="8">
         <v>27030</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="8">
         <v>2</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="8">
         <v>4</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="9">
         <v>12024</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="9">
         <v>1</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="9">
         <v>1</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="10">
+      <c r="B32" s="8">
         <v>51089</v>
       </c>
-      <c r="C32" s="10">
+      <c r="C32" s="8">
         <v>1</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="8">
         <v>1</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="9">
         <v>27342</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="9">
         <v>1</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="9">
         <v>1</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="8">
         <v>44643</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="8">
         <v>1</v>
       </c>
-      <c r="D34" s="10">
+      <c r="D34" s="8">
         <v>1</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="9">
         <v>2866</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="9">
         <v>1</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D35" s="9">
         <v>1</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B36" s="10">
+      <c r="B36" s="8">
         <v>2430</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="8">
         <v>1</v>
       </c>
-      <c r="D36" s="10">
+      <c r="D36" s="8">
         <v>1</v>
       </c>
-      <c r="E36" s="12" t="s">
-        <v>2966</v>
+      <c r="E36" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="9">
         <v>17561</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="9">
         <v>1</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D37" s="9">
         <v>1</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>347</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>1</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="8">
         <v>1</v>
       </c>
-      <c r="E38" s="12" t="s">
-        <v>2966</v>
+      <c r="E38" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="9">
         <v>22102</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="9">
         <v>1</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D39" s="9">
         <v>1</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B40" s="10">
+      <c r="B40" s="8">
         <v>21701</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C40" s="8">
         <v>1</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="8">
         <v>1</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="9">
         <v>23592</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="9">
         <v>1</v>
       </c>
-      <c r="D41" s="11">
+      <c r="D41" s="9">
         <v>1</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="8">
         <v>24701</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="8">
         <v>1</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="8">
         <v>1</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="9">
         <v>11122</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="9">
         <v>1</v>
       </c>
-      <c r="D43" s="11">
+      <c r="D43" s="9">
         <v>1</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="B44" s="10">
+      <c r="B44" s="8">
         <v>4911</v>
       </c>
-      <c r="C44" s="10">
+      <c r="C44" s="8">
         <v>1</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D44" s="8">
         <v>1</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="9">
         <v>31914</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="9">
         <v>1</v>
       </c>
-      <c r="D45" s="11">
+      <c r="D45" s="9">
         <v>2</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="8">
         <v>20147</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="8">
         <v>1</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="8">
         <v>2</v>
       </c>
-      <c r="E46" s="12" t="s">
-        <v>2966</v>
+      <c r="E46" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="9">
         <v>6758</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="9">
         <v>1</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D47" s="9">
         <v>2</v>
       </c>
-      <c r="E47" s="12" t="s">
-        <v>2966</v>
+      <c r="E47" s="10" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="B48" s="10">
+      <c r="B48" s="8">
         <v>25299</v>
       </c>
-      <c r="C48" s="10">
+      <c r="C48" s="8">
         <v>1</v>
       </c>
-      <c r="D48" s="10">
+      <c r="D48" s="8">
         <v>1</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="9">
         <v>12209</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="9">
         <v>1</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="9">
         <v>1</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="B50" s="10">
+      <c r="B50" s="8">
         <v>14124</v>
       </c>
-      <c r="C50" s="10">
+      <c r="C50" s="8">
         <v>1</v>
       </c>
-      <c r="D50" s="10">
+      <c r="D50" s="8">
         <v>1</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="9">
         <v>36958</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="9">
         <v>1</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D51" s="9">
         <v>1</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="B52" s="10">
+      <c r="B52" s="8">
         <v>13834</v>
       </c>
-      <c r="C52" s="10">
+      <c r="C52" s="8">
         <v>1</v>
       </c>
-      <c r="D52" s="10">
+      <c r="D52" s="8">
         <v>1</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="9">
         <v>763</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="9">
         <v>1</v>
       </c>
-      <c r="D53" s="11">
+      <c r="D53" s="9">
         <v>1</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B54" s="8">
         <v>23061</v>
       </c>
-      <c r="C54" s="10">
+      <c r="C54" s="8">
         <v>1</v>
       </c>
-      <c r="D54" s="10">
+      <c r="D54" s="8">
         <v>2</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
         <v>397</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="9">
         <v>19891</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="9">
         <v>1</v>
       </c>
-      <c r="D55" s="11">
+      <c r="D55" s="9">
         <v>2</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="B56" s="10">
+      <c r="B56" s="8">
         <v>5443</v>
       </c>
-      <c r="C56" s="10">
+      <c r="C56" s="8">
         <v>1</v>
       </c>
-      <c r="D56" s="10">
+      <c r="D56" s="8">
         <v>2</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="5" t="s">
         <v>454</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="9">
         <v>18683</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="9">
         <v>1</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="9">
         <v>2</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="3" t="s">
         <v>463</v>
       </c>
-      <c r="B58" s="10">
+      <c r="B58" s="8">
         <v>9849</v>
       </c>
-      <c r="C58" s="10">
+      <c r="C58" s="8">
         <v>1</v>
       </c>
-      <c r="D58" s="10">
+      <c r="D58" s="8">
         <v>2</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="B59" s="11">
+      <c r="B59" s="9">
         <v>5205</v>
       </c>
-      <c r="C59" s="11">
+      <c r="C59" s="9">
         <v>1</v>
       </c>
-      <c r="D59" s="11">
+      <c r="D59" s="9">
         <v>1</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="3" t="s">
         <v>511</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B60" s="8">
         <v>14023</v>
       </c>
-      <c r="C60" s="10">
+      <c r="C60" s="8">
         <v>1</v>
       </c>
-      <c r="D60" s="10">
+      <c r="D60" s="8">
         <v>1</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="5" t="s">
         <v>518</v>
       </c>
-      <c r="B61" s="11">
+      <c r="B61" s="9">
         <v>6935</v>
       </c>
-      <c r="C61" s="11">
+      <c r="C61" s="9">
         <v>1</v>
       </c>
-      <c r="D61" s="11">
+      <c r="D61" s="9">
         <v>2</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="3" t="s">
         <v>531</v>
       </c>
-      <c r="B62" s="10">
+      <c r="B62" s="8">
         <v>27276</v>
       </c>
-      <c r="C62" s="10">
+      <c r="C62" s="8">
         <v>1</v>
       </c>
-      <c r="D62" s="10">
+      <c r="D62" s="8">
         <v>1</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="5" t="s">
         <v>559</v>
       </c>
-      <c r="B63" s="11">
+      <c r="B63" s="9">
         <v>12507</v>
       </c>
-      <c r="C63" s="11">
+      <c r="C63" s="9">
         <v>1</v>
       </c>
-      <c r="D63" s="11">
+      <c r="D63" s="9">
         <v>2</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="3" t="s">
         <v>571</v>
       </c>
-      <c r="B64" s="10">
+      <c r="B64" s="8">
         <v>27838</v>
       </c>
-      <c r="C64" s="10">
+      <c r="C64" s="8">
         <v>1</v>
       </c>
-      <c r="D64" s="10">
+      <c r="D64" s="8">
         <v>2</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="5" t="s">
         <v>591</v>
       </c>
-      <c r="B65" s="11">
+      <c r="B65" s="9">
         <v>38991</v>
       </c>
-      <c r="C65" s="11">
+      <c r="C65" s="9">
         <v>1</v>
       </c>
-      <c r="D65" s="11">
+      <c r="D65" s="9">
         <v>2</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="3" t="s">
         <v>595</v>
       </c>
-      <c r="B66" s="10">
+      <c r="B66" s="8">
         <v>23196</v>
       </c>
-      <c r="C66" s="10">
+      <c r="C66" s="8">
         <v>1</v>
       </c>
-      <c r="D66" s="10">
+      <c r="D66" s="8">
         <v>2</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="B67" s="11">
+      <c r="B67" s="9">
         <v>18695</v>
       </c>
-      <c r="C67" s="11">
+      <c r="C67" s="9">
         <v>1</v>
       </c>
-      <c r="D67" s="11">
+      <c r="D67" s="9">
         <v>2</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="3" t="s">
         <v>617</v>
       </c>
-      <c r="B68" s="10">
+      <c r="B68" s="8">
         <v>11162</v>
       </c>
-      <c r="C68" s="10">
+      <c r="C68" s="8">
         <v>1</v>
       </c>
-      <c r="D68" s="10">
+      <c r="D68" s="8">
         <v>1</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="5" t="s">
         <v>635</v>
       </c>
-      <c r="B69" s="11">
+      <c r="B69" s="9">
         <v>14252</v>
       </c>
-      <c r="C69" s="11">
+      <c r="C69" s="9">
         <v>1</v>
       </c>
-      <c r="D69" s="11">
+      <c r="D69" s="9">
         <v>2</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="3" t="s">
         <v>639</v>
       </c>
-      <c r="B70" s="10">
+      <c r="B70" s="8">
         <v>14767</v>
       </c>
-      <c r="C70" s="10">
+      <c r="C70" s="8">
         <v>1</v>
       </c>
-      <c r="D70" s="10">
+      <c r="D70" s="8">
         <v>2</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="B71" s="11">
+      <c r="B71" s="9">
         <v>26388</v>
       </c>
-      <c r="C71" s="11">
+      <c r="C71" s="9">
         <v>1</v>
       </c>
-      <c r="D71" s="11">
+      <c r="D71" s="9">
         <v>2</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="3" t="s">
         <v>714</v>
       </c>
-      <c r="B72" s="10">
+      <c r="B72" s="8">
         <v>26443</v>
       </c>
-      <c r="C72" s="10">
+      <c r="C72" s="8">
         <v>1</v>
       </c>
-      <c r="D72" s="10">
+      <c r="D72" s="8">
         <v>2</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="5" t="s">
         <v>718</v>
       </c>
-      <c r="B73" s="11">
+      <c r="B73" s="9">
         <v>7195</v>
       </c>
-      <c r="C73" s="11">
+      <c r="C73" s="9">
         <v>1</v>
       </c>
-      <c r="D73" s="11">
+      <c r="D73" s="9">
         <v>2</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" s="3" t="s">
         <v>857</v>
       </c>
-      <c r="B74" s="10">
+      <c r="B74" s="8">
         <v>5335</v>
       </c>
-      <c r="C74" s="10">
+      <c r="C74" s="8">
         <v>1</v>
       </c>
-      <c r="D74" s="10">
+      <c r="D74" s="8">
         <v>2</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="5" t="s">
         <v>863</v>
       </c>
-      <c r="B75" s="11">
+      <c r="B75" s="9">
         <v>19273</v>
       </c>
-      <c r="C75" s="11">
+      <c r="C75" s="9">
         <v>1</v>
       </c>
-      <c r="D75" s="11">
+      <c r="D75" s="9">
         <v>2</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>2965</v>
+        <v>2961</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Täglich: 05.10.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan_daily.xlsx
+++ b/skipperplan_daily.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23521" uniqueCount="2966">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23519" uniqueCount="2964">
   <si>
     <t>Startdatum</t>
   </si>
@@ -948,7 +948,7 @@
     <t>MARTINE</t>
   </si>
   <si>
-    <t>Marlon S, Aaron B, Christof B, Gero L</t>
+    <t>Marlon S, Aaron B, Christof B, Gero L, Nadine Therese A</t>
   </si>
   <si>
     <t>16821</t>
@@ -1422,7 +1422,7 @@
     <t>16827</t>
   </si>
   <si>
-    <t>Christian N, Marlon S, Aaron B, Sarin G, Frank M, Viktoria B</t>
+    <t>Christian N, Marlon S, Aaron B, Sarin G, Frank M, Viktoria B, Nadine Therese A</t>
   </si>
   <si>
     <t>16826</t>
@@ -1455,7 +1455,7 @@
     <t>16719</t>
   </si>
   <si>
-    <t>Ralf B, Hendrik B, Julia H, Viktoria B</t>
+    <t>Ralf B, Hendrik B, Julia H, Viktoria B, Philipp K</t>
   </si>
   <si>
     <t>09.01.2027</t>
@@ -1476,7 +1476,7 @@
     <t>FARALLO</t>
   </si>
   <si>
-    <t>Bettina R, Marlon S, Aaron B, Philipp K, Lennart M</t>
+    <t>Bettina R, Marlon S, Aaron B, Philipp K, Lennart M, Nadine Therese A</t>
   </si>
   <si>
     <t>17335</t>
@@ -8896,12 +8896,6 @@
   </si>
   <si>
     <t>Neue Bewerbungen</t>
-  </si>
-  <si>
-    <t>Skipper geändert</t>
-  </si>
-  <si>
-    <t>(Kein Skipper)</t>
   </si>
   <si>
     <t>Neue Bewerbung(en)</t>
@@ -8958,7 +8952,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9003,12 +8997,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -9041,7 +9029,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -9064,13 +9052,10 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -13429,80 +13414,80 @@
       <c r="Z51" s="5"/>
     </row>
     <row r="52" spans="1:26">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D52" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="E52" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G52" s="6" t="s">
+      <c r="F52" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G52" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6">
+      <c r="H52" s="4"/>
+      <c r="I52" s="4">
         <v>8</v>
       </c>
-      <c r="J52" s="6">
-        <v>0</v>
-      </c>
-      <c r="K52" s="6" t="s">
+      <c r="J52" s="4">
+        <v>1</v>
+      </c>
+      <c r="K52" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="L52" s="6" t="s">
+      <c r="L52" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="M52" s="6" t="s">
+      <c r="M52" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="N52" s="6" t="s">
+      <c r="N52" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="O52" s="6" t="s">
+      <c r="O52" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="P52" s="6" t="s">
+      <c r="P52" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="Q52" s="6" t="s">
+      <c r="Q52" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="R52" s="6" t="s">
+      <c r="R52" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="S52" s="6" t="s">
+      <c r="S52" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="T52" s="6" t="s">
+      <c r="T52" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="U52" s="6" t="s">
+      <c r="U52" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="V52" s="6">
+      <c r="V52" s="4">
         <v>2017</v>
       </c>
-      <c r="W52" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="X52" s="6" t="s">
+      <c r="W52" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="X52" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="Y52" s="6" t="s">
+      <c r="Y52" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="Z52" s="6"/>
+      <c r="Z52" s="4"/>
     </row>
     <row r="53" spans="1:26">
       <c r="A53" s="5" t="s">
@@ -15741,7 +15726,7 @@
         <v>8</v>
       </c>
       <c r="J81" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K81" s="5" t="s">
         <v>166</v>
@@ -16365,7 +16350,7 @@
         <v>8</v>
       </c>
       <c r="J89" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K89" s="4" t="s">
         <v>166</v>
@@ -16835,7 +16820,7 @@
         <v>8</v>
       </c>
       <c r="J95" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K95" s="4" t="s">
         <v>166</v>
@@ -17227,7 +17212,7 @@
         <v>8</v>
       </c>
       <c r="J100" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K100" s="4" t="s">
         <v>166</v>
@@ -18087,7 +18072,7 @@
         <v>8</v>
       </c>
       <c r="J111" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K111" s="4" t="s">
         <v>166</v>
@@ -20561,7 +20546,7 @@
         <v>8</v>
       </c>
       <c r="J143" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K143" s="4" t="s">
         <v>166</v>
@@ -23717,7 +23702,7 @@
         <v>9</v>
       </c>
       <c r="J184" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K184" s="4" t="s">
         <v>166</v>
@@ -91270,103 +91255,99 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="3" t="s">
         <v>2957</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>2958</v>
-      </c>
-      <c r="I2" s="8"/>
+      <c r="B2" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>2957</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>2958</v>
-      </c>
-      <c r="I3" s="8"/>
+      <c r="B3" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="3" t="s">
-        <v>2959</v>
+        <v>2957</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>299</v>
+        <v>398</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>390</v>
+        <v>462</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
-        <v>309</v>
+        <v>402</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3" t="s">
-        <v>282</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>2959</v>
+        <v>2957</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>299</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>696</v>
+        <v>462</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>750</v>
+        <v>477</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="G5" s="3"/>
+        <v>482</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>478</v>
+      </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3" t="s">
-        <v>282</v>
+        <v>1013</v>
       </c>
     </row>
   </sheetData>
@@ -91392,1087 +91373,1087 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2958</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2959</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2960</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2961</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2962</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2963</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>14111</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>5</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>6</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>2964</v>
+      <c r="E2" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="10">
         <v>6429</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="10">
         <v>4</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="10">
         <v>6</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>2964</v>
+      <c r="E3" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>26133</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>4</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>6</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <v>951</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="10">
         <v>4</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="10">
         <v>6</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>2964</v>
+      <c r="E5" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>26767</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>4</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>8</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <v>13035</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <v>3</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="10">
         <v>4</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>2964</v>
+      <c r="E7" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>13045</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="8">
         <v>3</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="8">
         <v>5</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <v>28325</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="10">
         <v>3</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="10">
         <v>4</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>2964</v>
+      <c r="E9" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>27428</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>3</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <v>13707</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="10">
         <v>3</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="10">
         <v>3</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>2964</v>
+      <c r="E11" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>38409</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>3</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>6</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <v>7022</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="10">
         <v>2</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="10">
         <v>2</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>2964</v>
+      <c r="E13" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>25998</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>2</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <v>27634</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="10">
         <v>2</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="10">
         <v>2</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>9630</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>2</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="8">
         <v>2</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <v>27191</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="10">
         <v>2</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="10">
         <v>2</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>27871</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>2</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>2</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <v>17277</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="10">
         <v>2</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="10">
         <v>4</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>2964</v>
+      <c r="E19" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>2257</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>2</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>4</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <v>27366</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="10">
         <v>2</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <v>4</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="8">
         <v>25583</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="8">
         <v>2</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="8">
         <v>4</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <v>15339</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="10">
         <v>2</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <v>4</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="8">
         <v>27408</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="8">
         <v>2</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="8">
         <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="5" t="s">
         <v>576</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="10">
         <v>27030</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="10">
         <v>2</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <v>4</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="8">
         <v>3641</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="8">
         <v>1</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>1</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="10">
         <v>3223</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="10">
         <v>1</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="10">
         <v>1</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>22825</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="8">
         <v>1</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="8">
         <v>1</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="10">
         <v>11122</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="10">
         <v>1</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="10">
         <v>1</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="8">
         <v>4911</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="8">
         <v>1</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="8">
         <v>1</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="10">
         <v>31914</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="10">
         <v>1</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="10">
         <v>2</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="8">
         <v>20147</v>
       </c>
-      <c r="C32" s="9">
+      <c r="C32" s="8">
         <v>1</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="8">
         <v>2</v>
       </c>
-      <c r="E32" s="10" t="s">
-        <v>2964</v>
+      <c r="E32" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="10">
         <v>6758</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="10">
         <v>1</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="10">
         <v>2</v>
       </c>
-      <c r="E33" s="10" t="s">
-        <v>2964</v>
+      <c r="E33" s="9" t="s">
+        <v>2962</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="8">
         <v>25299</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="8">
         <v>1</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="8">
         <v>1</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="10">
         <v>12209</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="10">
         <v>1</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D35" s="10">
         <v>1</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <v>14124</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="8">
         <v>1</v>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="8">
         <v>1</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="10">
         <v>36958</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="10">
         <v>1</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D37" s="10">
         <v>1</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="8">
         <v>13834</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="8">
         <v>1</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="8">
         <v>1</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="10">
         <v>763</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="10">
         <v>1</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D39" s="10">
         <v>1</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="8">
         <v>23061</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="8">
         <v>1</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="8">
         <v>2</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="10">
         <v>19891</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="10">
         <v>1</v>
       </c>
-      <c r="D41" s="11">
+      <c r="D41" s="10">
         <v>2</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="8">
         <v>5443</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="8">
         <v>1</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="8">
         <v>2</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="10">
         <v>5688</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="10">
         <v>1</v>
       </c>
-      <c r="D43" s="11">
+      <c r="D43" s="10">
         <v>1</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="8">
         <v>18683</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="8">
         <v>1</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="8">
         <v>2</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="10">
         <v>9849</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="10">
         <v>1</v>
       </c>
-      <c r="D45" s="11">
+      <c r="D45" s="10">
         <v>2</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="8">
         <v>5205</v>
       </c>
-      <c r="C46" s="9">
+      <c r="C46" s="8">
         <v>1</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="8">
         <v>1</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="10">
         <v>14023</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="10">
         <v>1</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D47" s="10">
         <v>1</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="3" t="s">
         <v>437</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="8">
         <v>6935</v>
       </c>
-      <c r="C48" s="9">
+      <c r="C48" s="8">
         <v>1</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="8">
         <v>2</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="5" t="s">
         <v>450</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="10">
         <v>27276</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="10">
         <v>1</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="10">
         <v>1</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="3" t="s">
         <v>478</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="8">
         <v>12507</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C50" s="8">
         <v>1</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50" s="8">
         <v>2</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="5" t="s">
         <v>490</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="10">
         <v>27838</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="10">
         <v>1</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D51" s="10">
         <v>2</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="3" t="s">
         <v>510</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="8">
         <v>38991</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52" s="8">
         <v>1</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="8">
         <v>2</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="5" t="s">
         <v>514</v>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="10">
         <v>23196</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="10">
         <v>1</v>
       </c>
-      <c r="D53" s="11">
+      <c r="D53" s="10">
         <v>2</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="3" t="s">
         <v>525</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="8">
         <v>18695</v>
       </c>
-      <c r="C54" s="9">
+      <c r="C54" s="8">
         <v>1</v>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="8">
         <v>2</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="10">
         <v>11162</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="10">
         <v>1</v>
       </c>
-      <c r="D55" s="11">
+      <c r="D55" s="10">
         <v>1</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="3" t="s">
         <v>547</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="8">
         <v>38249</v>
       </c>
-      <c r="C56" s="9">
+      <c r="C56" s="8">
         <v>1</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="8">
         <v>2</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="10">
         <v>14252</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="10">
         <v>1</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="10">
         <v>2</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="3" t="s">
         <v>560</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="8">
         <v>14767</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="8">
         <v>1</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="8">
         <v>2</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="5" t="s">
         <v>590</v>
       </c>
-      <c r="B59" s="11">
+      <c r="B59" s="10">
         <v>26388</v>
       </c>
-      <c r="C59" s="11">
+      <c r="C59" s="10">
         <v>1</v>
       </c>
-      <c r="D59" s="11">
+      <c r="D59" s="10">
         <v>2</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="3" t="s">
         <v>637</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="8">
         <v>26443</v>
       </c>
-      <c r="C60" s="9">
+      <c r="C60" s="8">
         <v>1</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="8">
         <v>2</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="5" t="s">
         <v>641</v>
       </c>
-      <c r="B61" s="11">
+      <c r="B61" s="10">
         <v>7195</v>
       </c>
-      <c r="C61" s="11">
+      <c r="C61" s="10">
         <v>1</v>
       </c>
-      <c r="D61" s="11">
+      <c r="D61" s="10">
         <v>2</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="3" t="s">
         <v>676</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="8">
         <v>17056</v>
       </c>
-      <c r="C62" s="9">
+      <c r="C62" s="8">
         <v>1</v>
       </c>
-      <c r="D62" s="9">
+      <c r="D62" s="8">
         <v>2</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="5" t="s">
         <v>782</v>
       </c>
-      <c r="B63" s="11">
+      <c r="B63" s="10">
         <v>5335</v>
       </c>
-      <c r="C63" s="11">
+      <c r="C63" s="10">
         <v>1</v>
       </c>
-      <c r="D63" s="11">
+      <c r="D63" s="10">
         <v>2</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="3" t="s">
         <v>788</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="8">
         <v>19273</v>
       </c>
-      <c r="C64" s="9">
+      <c r="C64" s="8">
         <v>1</v>
       </c>
-      <c r="D64" s="9">
+      <c r="D64" s="8">
         <v>2</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>2965</v>
+        <v>2963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Täglich: 12.10.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan_daily.xlsx
+++ b/skipperplan_daily.xlsx
@@ -1503,7 +1503,7 @@
     <t>16837</t>
   </si>
   <si>
-    <t>Fabio M, Marlon S, Jonas H, Aaron B, Johanna S, Ilga P</t>
+    <t>Fabio M, Marlon S, Jonas H, Aaron B, Johanna S, Ilga P, Lennart M</t>
   </si>
   <si>
     <t>16838</t>
@@ -1710,7 +1710,7 @@
     <t>16808</t>
   </si>
   <si>
-    <t>Fabio M, Marlon S, Stefan D, Paul S, Mareike W, Aaron B, Christoph C, Ilga P</t>
+    <t>Fabio M, Marlon S, Stefan D, Paul S, Mareike W, Aaron B, Christoph C, Ilga P, Lennart M</t>
   </si>
   <si>
     <t>16809</t>
@@ -2073,7 +2073,7 @@
     <t>16853</t>
   </si>
   <si>
-    <t>Bettina R, Marlon S, Viktoria B</t>
+    <t>Bettina R, Marlon S, Viktoria B, Lennart M</t>
   </si>
   <si>
     <t>17281</t>
@@ -2091,7 +2091,7 @@
     <t>16849</t>
   </si>
   <si>
-    <t>Jens B, Ralf B, Tim G, Bettina R, Marlon S, Mirco K, Viktoria B</t>
+    <t>Jens B, Ralf B, Tim G, Bettina R, Marlon S, Mirco K, Viktoria B, Lennart M</t>
   </si>
   <si>
     <t>16850</t>
@@ -2238,7 +2238,7 @@
     <t>16810</t>
   </si>
   <si>
-    <t>Tim G, Marlon S, Marlena G</t>
+    <t>Tim G, Marlon S, Marlena G, Lennart M</t>
   </si>
   <si>
     <t>16811</t>
@@ -12667,7 +12667,7 @@
         <v>12</v>
       </c>
       <c r="J42" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K42" s="3" t="s">
         <v>198</v>
@@ -14555,7 +14555,7 @@
         <v>8</v>
       </c>
       <c r="J66" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K66" s="4" t="s">
         <v>198</v>
@@ -15025,7 +15025,7 @@
         <v>8</v>
       </c>
       <c r="J72" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K72" s="4" t="s">
         <v>198</v>
@@ -15263,7 +15263,7 @@
         <v>8</v>
       </c>
       <c r="J75" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K75" s="5" t="s">
         <v>198</v>
@@ -16123,7 +16123,7 @@
         <v>8</v>
       </c>
       <c r="J86" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K86" s="3" t="s">
         <v>198</v>
@@ -17899,7 +17899,7 @@
         <v>12</v>
       </c>
       <c r="J109" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K109" s="4" t="s">
         <v>198</v>
@@ -18827,7 +18827,7 @@
         <v>8</v>
       </c>
       <c r="J121" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K121" s="4" t="s">
         <v>198</v>
@@ -22291,7 +22291,7 @@
         <v>8</v>
       </c>
       <c r="J166" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K166" s="4" t="s">
         <v>198</v>
@@ -24067,7 +24067,7 @@
         <v>8</v>
       </c>
       <c r="J189" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K189" s="5" t="s">
         <v>198</v>
@@ -91369,21 +91369,19 @@
         <v>213</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>383</v>
+        <v>400</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>400</v>
+        <v>489</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>157</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3" t="s">
-        <v>157</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -91391,22 +91389,24 @@
         <v>2960</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>239</v>
+        <v>271</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>651</v>
+        <v>548</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>652</v>
+        <v>549</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="G3" s="3"/>
+        <v>437</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
-        <v>466</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -91414,22 +91414,22 @@
         <v>2960</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>319</v>
+        <v>213</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>643</v>
+        <v>623</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>623</v>
+        <v>679</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
-        <v>323</v>
+        <v>406</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3" t="s">
-        <v>659</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -91437,22 +91437,22 @@
         <v>2960</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>319</v>
+        <v>271</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>623</v>
+        <v>675</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>675</v>
+        <v>734</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>323</v>
+        <v>437</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3" t="s">
-        <v>659</v>
+        <v>1564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>